<commit_message>
Merge user's Mar-25 sheet into state table: max of awarded/deployed per state; add Haryana
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Metering_Statewise_Latest.xlsx
+++ b/Smart_Metering_Statewise_Latest.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">State-wise Smart Meters, mn nos — latest available (as on Aug-2026)</t>
   </si>
@@ -79,22 +79,25 @@
     <t xml:space="preserve">Andhra Pradesh</t>
   </si>
   <si>
-    <t xml:space="preserve">Total (13 states)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sanctioned &amp; Awarded: official RDSS state table, Rajya Sabha reply 10-Feb-2025 (via data.gov.in API) — the latest full official filing; no newer state-wise award filing exists publicly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deployed (latest reported): Maharashtra 12.5 (Jul-26, MSEDCL &gt;1.25 crore); Bihar 9.2 (01-Jul-26); UP 8.5 (Jun-26, ~85 lakh); Gujarat 2.09 (15-Jul-26, 20.94 lakh); Assam 3.28 (Mar-25); all others as per 10-Feb-2025 official reply — no newer public figure found.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">* Bihar: all schemes (state scheme + RDSS); its RDSS-only sanction is 2.61 mn. Sanction/award 17.21 mn per Mar-25 reporting (172.09 lakh, fully awarded).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tamil Nadu: tender live (Genus call, 19-May-26), award pending. Punjab: LoA issued to TCIL 30-Jan-26 but agreement unsigned (Jul-26) — shown as not awarded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yet to be awarded = MAX(0, Sanctioned - Awarded). All-India context: sanctioned 203.4 (RDSS), tendered ~156 (Genus 19-May-26), installed 72.4 (30-Jun-26, Parliament).</t>
+    <t xml:space="preserve">Haryana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total (14 states)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awarded &amp; Deployed = higher of: (a) official RDSS state table, Rajya Sabha reply 10-Feb-2025 (data.gov.in); (b) user's dashboard sheet as on 04-Mar-2025; (c) latest dated 2026 reports.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From (c): Maharashtra deployed 12.5 (Jul-26, MSEDCL &gt;1.25 crore); Bihar 9.2 (01-Jul-26); UP 8.5 (Jun-26); Gujarat 2.09 (15-Jul-26); Assam 3.28 (Mar-25).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From (b): UP awarded 31.00; Rajasthan 15.00/1.00; MP 6.00/2.00; Punjab 1.00/1.00; Haryana 1.00/1.00/1.00 (Haryana absent from RDSS filing).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* Bihar on all-schemes basis (RDSS-only sanction 2.61). UP awarded exceeds RDSS sanction as it includes non-RDSS UP awards (UP total sanction incl. non-RDSS ~31).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yet to be awarded = MAX(0, Sanctioned - Awarded). All-India context: sanctioned 203.4 RDSS (222 all schemes), tendered ~156 (Genus call 19-May-26), installed 72.4 (30-Jun-26, Parliament).</t>
   </si>
 </sst>
 </file>
@@ -524,7 +527,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F23"/>
+  <dimension ref="B1:F24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -581,7 +584,7 @@
         <v>28.53</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>28.53</v>
+        <v>31</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>8.5</v>
@@ -671,10 +674,10 @@
         <v>14.74</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>14.75</v>
+        <v>15</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">MAX(0,C10-D10)</f>
@@ -689,14 +692,14 @@
         <v>13.43</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>5.49</v>
+        <v>6</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>1.37</v>
+        <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">MAX(0,C11-D11)</f>
-        <v>7.94</v>
+        <v>7.43</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -725,14 +728,14 @@
         <v>8.98</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
         <f aca="false">MAX(0,C13-D13)</f>
-        <v>8.98</v>
+        <v>7.98</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -790,34 +793,43 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="7" t="n">
-        <f aca="false">SUM(C4:C16)</f>
-        <v>207.14</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <f aca="false">SUM(D4:D16)</f>
-        <v>126.53</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <f aca="false">SUM(E4:E16)</f>
-        <v>39.13</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <f aca="false">SUM(F4:F16)</f>
-        <v>83.23</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="8" t="s">
+      <c r="C17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <f aca="false">MAX(0,C17-D17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
+      <c r="C18" s="7" t="n">
+        <f aca="false">SUM(C4:C17)</f>
+        <v>208.14</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <f aca="false">SUM(D4:D17)</f>
+        <v>131.76</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <f aca="false">SUM(E4:E17)</f>
+        <v>42.75</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <f aca="false">SUM(F4:F17)</f>
+        <v>81.72</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
@@ -855,13 +867,22 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
+    <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="B19:F19"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B24:F24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Update deployed to official 30-Jun-2026 state-wise figures (RS reply 27-Jul-2026)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Metering_Statewise_Latest.xlsx
+++ b/Smart_Metering_Statewise_Latest.xlsx
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
-  <si>
-    <t xml:space="preserve">State-wise Smart Meters, mn nos — latest available (as on Aug-2026)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+  <si>
+    <t xml:space="preserve">State-wise Smart Meters, mn nos — Deployed as on 30-Jun-2026 (official)</t>
   </si>
   <si>
     <t xml:space="preserve">State</t>
@@ -79,25 +79,34 @@
     <t xml:space="preserve">Andhra Pradesh</t>
   </si>
   <si>
+    <t xml:space="preserve">Himachal Pradesh</t>
+  </si>
+  <si>
     <t xml:space="preserve">Haryana</t>
   </si>
   <si>
-    <t xml:space="preserve">Total (14 states)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awarded &amp; Deployed = higher of: (a) official RDSS state table, Rajya Sabha reply 10-Feb-2025 (data.gov.in); (b) user's dashboard sheet as on 04-Mar-2025; (c) latest dated 2026 reports.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From (c): Maharashtra deployed 12.5 (Jul-26, MSEDCL &gt;1.25 crore); Bihar 9.2 (01-Jul-26); UP 8.5 (Jun-26); Gujarat 2.09 (15-Jul-26); Assam 3.28 (Mar-25).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From (b): UP awarded 31.00; Rajasthan 15.00/1.00; MP 6.00/2.00; Punjab 1.00/1.00; Haryana 1.00/1.00/1.00 (Haryana absent from RDSS filing).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">* Bihar on all-schemes basis (RDSS-only sanction 2.61). UP awarded exceeds RDSS sanction as it includes non-RDSS UP awards (UP total sanction incl. non-RDSS ~31).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yet to be awarded = MAX(0, Sanctioned - Awarded). All-India context: sanctioned 203.4 RDSS (222 all schemes), tendered ~156 (Genus call 19-May-26), installed 72.4 (30-Jun-26, Parliament).</t>
+    <t xml:space="preserve">Total (15 states)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All India (RDSS, official 30-Jun-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All India (all schemes, 30-Jun-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deployed: official state-wise table, Rajya Sabha reply dated 27-Jul-2026, data as on 30-Jun-2026 (RDSS: consumer+DT+feeder). Top-10 states as published; WB/TN/Kerala/Punjab/Haryana from other sources as noted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Official 30-Jun-26 installed (lakh): Maharashtra 129.73, UP 97.54, Assam 55.44, Gujarat 52.01, Rajasthan 47.59, Chhattisgarh 42.23, MP 41.90, AP 32.80, Bihar(RDSS) 23.02, HP 10.06; top-10 total 532.33; rest of India 40.99; grand total 573.32.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* Bihar shown all-schemes: 9.20 (01-Jul-26 reporting; RDSS-only official = 2.30). Punjab &amp; Haryana deployed 1.00 from user's 04-Mar-25 sheet (official RDSS = 0 / not sanctioned) — retained per max rule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awarded: no official state-wise award filing after 10-Feb-2025; column = higher of that filing and user's 04-Mar-25 sheet. All-India awarded/tendered ~156 (Genus Q4FY26 call, 19-May-26).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yet to be awarded = MAX(0, Sanctioned - Awarded). Reconciliation: RDSS 57.33 + non-RDSS (~15.1, mostly Bihar state scheme, UP legacy, TN/Delhi NSGM) = 72.4 all-India.</t>
   </si>
 </sst>
 </file>
@@ -238,7 +247,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -268,6 +277,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -527,11 +540,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F24"/>
+  <dimension ref="B1:F27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
   </cols>
@@ -587,7 +600,7 @@
         <v>31</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>8.5</v>
+        <v>9.75</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">MAX(0,C5-D5)</f>
@@ -605,7 +618,7 @@
         <v>25.27</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>12.5</v>
+        <v>12.97</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">MAX(0,C6-D6)</f>
@@ -659,7 +672,7 @@
         <v>11.07</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>2.09</v>
+        <v>5.2</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">MAX(0,C9-D9)</f>
@@ -677,7 +690,7 @@
         <v>15</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1</v>
+        <v>4.76</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">MAX(0,C10-D10)</f>
@@ -695,7 +708,7 @@
         <v>6</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>2</v>
+        <v>4.19</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">MAX(0,C11-D11)</f>
@@ -749,7 +762,7 @@
         <v>6.56</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>3.28</v>
+        <v>5.54</v>
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">MAX(0,C14-D14)</f>
@@ -767,7 +780,7 @@
         <v>7.35</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1.05</v>
+        <v>4.22</v>
       </c>
       <c r="F15" s="5" t="n">
         <f aca="false">MAX(0,C15-D15)</f>
@@ -785,7 +798,7 @@
         <v>5.98</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.82</v>
+        <v>3.28</v>
       </c>
       <c r="F16" s="5" t="n">
         <f aca="false">MAX(0,C16-D16)</f>
@@ -797,92 +810,141 @@
         <v>19</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1</v>
+        <v>2.84</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>1</v>
+        <v>0.93</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">MAX(0,C17-D17)</f>
-        <v>0</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="7" t="n">
-        <f aca="false">SUM(C4:C17)</f>
-        <v>208.14</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <f aca="false">SUM(D4:D17)</f>
-        <v>131.76</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <f aca="false">SUM(E4:E17)</f>
-        <v>42.75</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <f aca="false">SUM(F4:F17)</f>
-        <v>81.72</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="8" t="s">
+      <c r="C18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <f aca="false">MAX(0,C18-D18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="8"/>
+      <c r="C19" s="7" t="n">
+        <f aca="false">SUM(C4:C18)</f>
+        <v>210.98</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <f aca="false">SUM(D4:D18)</f>
+        <v>132.69</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <f aca="false">SUM(E4:E18)</f>
+        <v>62.43</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <f aca="false">SUM(F4:F18)</f>
+        <v>83.63</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>203.39</v>
+      </c>
       <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
+      <c r="E20" s="4" t="n">
+        <v>57.33</v>
+      </c>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-    </row>
-    <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="8" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-    </row>
-    <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
+      <c r="C21" s="4" t="n">
+        <v>222</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>72.4</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <f aca="false">MAX(0,C21-D21)</f>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-    </row>
-    <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8" t="s">
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+    </row>
+    <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+    </row>
+    <row r="27" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:F22"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Merge NSGM Mar-2026 dashboard data: sanctions to 229.8 mn, fill Punjab/WB/Kerala/TN deployed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168WxZRzFr3YzWSe68Nt1CM
</commit_message>
<xml_diff>
--- a/Smart_Metering_Statewise_Latest.xlsx
+++ b/Smart_Metering_Statewise_Latest.xlsx
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
-  <si>
-    <t xml:space="preserve">State-wise Smart Meters, mn nos — Deployed as on 30-Jun-2026 (official)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+  <si>
+    <t xml:space="preserve">State-wise Smart Meters, mn nos — as on Aug-2026 (all schemes)</t>
   </si>
   <si>
     <t xml:space="preserve">State</t>
@@ -40,19 +40,19 @@
     <t xml:space="preserve">Yet to be awarded</t>
   </si>
   <si>
+    <t xml:space="preserve">Uttar Pradesh</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tamil Nadu</t>
   </si>
   <si>
-    <t xml:space="preserve">Uttar Pradesh</t>
-  </si>
-  <si>
     <t xml:space="preserve">Maharashtra</t>
   </si>
   <si>
     <t xml:space="preserve">West Bengal</t>
   </si>
   <si>
-    <t xml:space="preserve">Bihar*</t>
+    <t xml:space="preserve">Bihar</t>
   </si>
   <si>
     <t xml:space="preserve">Gujarat</t>
@@ -88,25 +88,28 @@
     <t xml:space="preserve">Total (15 states)</t>
   </si>
   <si>
-    <t xml:space="preserve">All India (RDSS, official 30-Jun-26)</t>
+    <t xml:space="preserve">All India (NSGM all schemes, 31-Mar-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All India (RDSS only, 30-Jun-26)</t>
   </si>
   <si>
     <t xml:space="preserve">All India (all schemes, 30-Jun-26)</t>
   </si>
   <si>
-    <t xml:space="preserve">Deployed: official state-wise table, Rajya Sabha reply dated 27-Jul-2026, data as on 30-Jun-2026 (RDSS: consumer+DT+feeder). Top-10 states as published; WB/TN/Kerala/Punjab/Haryana from other sources as noted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Official 30-Jun-26 installed (lakh): Maharashtra 129.73, UP 97.54, Assam 55.44, Gujarat 52.01, Rajasthan 47.59, Chhattisgarh 42.23, MP 41.90, AP 32.80, Bihar(RDSS) 23.02, HP 10.06; top-10 total 532.33; rest of India 40.99; grand total 573.32.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">* Bihar shown all-schemes: 9.20 (01-Jul-26 reporting; RDSS-only official = 2.30). Punjab &amp; Haryana deployed 1.00 from user's 04-Mar-25 sheet (official RDSS = 0 / not sanctioned) — retained per max rule.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awarded: no official state-wise award filing after 10-Feb-2025; column = higher of that filing and user's 04-Mar-25 sheet. All-India awarded/tendered ~156 (Genus Q4FY26 call, 19-May-26).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yet to be awarded = MAX(0, Sanctioned - Awarded). Reconciliation: RDSS 57.33 + non-RDSS (~15.1, mostly Bihar state scheme, UP legacy, TN/Delhi NSGM) = 72.4 all-India.</t>
+    <t xml:space="preserve">Sanctioned: NSGM dashboard 'Approved' as of Mar-2026 (The Secretariat infographic, all schemes; overall 2298.06 lakh = 229.81 mn incl. consumer 2242.80 + DT 53.20 + feeder 2.07 lakh) for its top-10 states; official RDSS filing for Assam/Chhattisgarh/AP/HP; Haryana per user sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deployed = newest of: NSGM Mar-26 (Punjab 20.76 L, WB 5.74 L, Kerala 1.73 L, TN 1.29 L); official RS reply 27-Jul-26 as on 30-Jun-26 (Maharashtra 129.73 L, UP 97.54 L, Assam 55.44 L, Gujarat 52.01 L, Rajasthan 47.59 L, Chhattisgarh 42.23 L, MP 41.90 L, AP 32.80 L, HP 10.06 L); Bihar 92 L (01-Jul-26 reporting).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awarded: no official state-wise award filing after 10-Feb-2025; column = higher of that filing and user's 04-Mar-25 sheet. Punjab shows deployed (2.08) &gt; awarded (1.00) because its NSGM-era installs predate the pending RDSS award (LoA to TCIL 30-Jan-26 unsigned). All-India awarded/tendered ~156 (Genus call 19-May-26).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NSGM Mar-26 install progress %: Bihar 50.5, Maharashtra 37.7, MP 27.5, UP 27.2, Gujarat 23.5, Rajasthan 22.4, Punjab 18.5, WB 2.7, Kerala 1.3, TN 0.4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yet to be awarded = MAX(0, Sanctioned - Awarded). Reconciliation: RDSS 57.33 (Jun-26) + non-RDSS ~15.1 = 72.4 all-India; NSGM all-schemes 58.34 (Mar-26) grew to 72.4 by Jun-26.</t>
   </si>
 </sst>
 </file>
@@ -540,11 +543,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F27"/>
+  <dimension ref="B1:F28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
   </cols>
@@ -576,17 +579,17 @@
         <v>6</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>30.49</v>
+        <v>30.9</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.13</v>
+        <v>9.75</v>
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">MAX(0,C4-D4)</f>
-        <v>30.49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -594,17 +597,17 @@
         <v>7</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>28.53</v>
+        <v>30.1</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>9.75</v>
+        <v>0.13</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">MAX(0,C5-D5)</f>
-        <v>0</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -612,7 +615,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>24</v>
+        <v>23.5</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>25.27</v>
@@ -630,17 +633,17 @@
         <v>9</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>21.04</v>
+        <v>21.2</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>4.03</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.18</v>
+        <v>0.57</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">MAX(0,C7-D7)</f>
-        <v>17.01</v>
+        <v>17.17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -648,7 +651,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>17.21</v>
+        <v>17.2</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>17.21</v>
@@ -666,7 +669,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>16.79</v>
+        <v>16.5</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>11.07</v>
@@ -676,7 +679,7 @@
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">MAX(0,C9-D9)</f>
-        <v>5.72</v>
+        <v>5.43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -684,7 +687,7 @@
         <v>12</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>14.74</v>
+        <v>14.9</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>15</v>
@@ -702,7 +705,7 @@
         <v>13</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>13.43</v>
+        <v>13.4</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>6</v>
@@ -712,7 +715,7 @@
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">MAX(0,C11-D11)</f>
-        <v>7.43</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -720,17 +723,17 @@
         <v>14</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>13.38</v>
+        <v>13.2</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>0.29</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">MAX(0,C12-D12)</f>
-        <v>13.09</v>
+        <v>12.91</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -738,17 +741,17 @@
         <v>15</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>8.98</v>
+        <v>11.2</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>1</v>
+        <v>2.08</v>
       </c>
       <c r="F13" s="5" t="n">
         <f aca="false">MAX(0,C13-D13)</f>
-        <v>7.98</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -847,7 +850,7 @@
       </c>
       <c r="C19" s="7" t="n">
         <f aca="false">SUM(C4:C18)</f>
-        <v>210.98</v>
+        <v>214.49</v>
       </c>
       <c r="D19" s="7" t="n">
         <f aca="false">SUM(D4:D18)</f>
@@ -855,11 +858,11 @@
       </c>
       <c r="E19" s="7" t="n">
         <f aca="false">SUM(E4:E18)</f>
-        <v>62.43</v>
+        <v>64.07</v>
       </c>
       <c r="F19" s="7" t="n">
         <f aca="false">SUM(F4:F18)</f>
-        <v>83.63</v>
+        <v>85.12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -867,11 +870,11 @@
         <v>22</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>203.39</v>
+        <v>229.81</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="4" t="n">
-        <v>57.33</v>
+        <v>58.34</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -880,29 +883,33 @@
         <v>23</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>222</v>
-      </c>
-      <c r="D21" s="4" t="n">
+        <v>203.39</v>
+      </c>
+      <c r="D21" s="8"/>
+      <c r="E21" s="4" t="n">
+        <v>57.33</v>
+      </c>
+      <c r="F21" s="8"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>229.81</v>
+      </c>
+      <c r="D22" s="4" t="n">
         <v>156</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E22" s="4" t="n">
         <v>72.4</v>
       </c>
-      <c r="F21" s="5" t="n">
-        <f aca="false">MAX(0,C21-D21)</f>
-        <v>66</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-    </row>
-    <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F22" s="5" t="n">
+        <f aca="false">MAX(0,C22-D22)</f>
+        <v>73.81</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="9" t="s">
         <v>25</v>
       </c>
@@ -911,7 +918,7 @@
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="9" t="s">
         <v>26</v>
       </c>
@@ -920,7 +927,7 @@
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="9" t="s">
         <v>27</v>
       </c>
@@ -929,7 +936,7 @@
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="9" t="s">
         <v>28</v>
       </c>
@@ -938,13 +945,22 @@
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
     </row>
+    <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:F28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>